<commit_message>
Verifica settimanale: 181 duplicati marcati, 90 upgrade doppio controllo
- Deduplica globale su 340 file (2545 righe), corretti 3 bug scoperti
  prima del commit: foglio "Scartati" letto come attivo invece di
  "Distributori" in 8 file storici; placeholder "n.d." in sito_web
  trattato come dominio reale; domini di piattaforme condivise
  (mall.lapasar.com, facebook.com, karcher.com/kaercher.com) usati
  per accorpare erroneamente aziende indipendenti.
- Doppio controllo via WebSearch (9 agenti paralleli) su 114 righe
  "DA VERIFICARE UMANAMENTE" nei 46 file nuovi: 90 promosse a
  "VERIFICATA AI - doppio controllo", 24 lasciate invariate per
  esito non confermato o settore incoerente.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014bsWXkinKKsa91GXsTxgBM
</commit_message>
<xml_diff>
--- a/output/2026-09-14_00_Croazia_Primorsko-goranska_Utensilerie_e_Macchine_Utensili.xlsx
+++ b/output/2026-09-14_00_Croazia_Primorsko-goranska_Utensilerie_e_Macchine_Utensili.xlsx
@@ -775,7 +775,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Grossista utensili industriali, fissaggi, attrezzature officina</t>
+          <t>Grossista utensili industriali, fissaggi, attrezzature officina [DUPLICATO — vedi anche: 2026-09-13_02_Croazia_Varazdinska_Metalworking_Lavorazioni_Metalliche.xlsx]</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -817,7 +817,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Grossista utensili industriali, fissaggi, attrezzature officina. Sede distinta da Viškovo</t>
+          <t>Grossista utensili industriali, fissaggi, attrezzature officina. Sede distinta da Viškovo [DUPLICATO — vedi anche: 2026-09-13_02_Croazia_Varazdinska_Metalworking_Lavorazioni_Metalliche.xlsx]</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">

</xml_diff>